<commit_message>
📋 TA Scan 2026-03-20 14:54 UTC — profilo: hr-roma
</commit_message>
<xml_diff>
--- a/output/TA_Monitor_Selezione_HR_Roma_2026-03-20.xlsx
+++ b/output/TA_Monitor_Selezione_HR_Roma_2026-03-20.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Posizioni" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Posizioni'!$A$1:$I$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Posizioni'!$A$1:$I$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I114"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -497,12 +497,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Project Analyst - Ecosistema Futuro</t>
+          <t>Ingegnere Civile</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>RONZONI GROUP STP STL SB</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -520,24 +520,24 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=9794cfdbbd68de5e</t>
+          <t>https://it.indeed.com/viewjob?jk=59a010eab9898993</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Addetto/a Risorse Umane – Selezione e Formazione</t>
+          <t>Impiegato/a Ufficio Risorse Umane - Settore GDO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EmmeBi Group</t>
+          <t>tecno-system</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -555,7 +555,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4387394112</t>
+          <t>https://www.linkedin.com/jobs/view/4388356588</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -563,12 +563,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Addetto/a Risorse Umane - HR</t>
+          <t>HR Recruiter Assistant L.68/99 - Categoria Protetta Part Time</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>To Be Service srl</t>
+          <t>BIP</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -586,24 +586,20 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4387120451</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4388343180</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Operatore Elettrotermico</t>
+          <t>HR Business Partner, EU One PXT</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -616,29 +612,33 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=c55d6bbd098a4b74</t>
+          <t>https://it.indeed.com/viewjob?jk=33e5087195e907bd</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Commerciali</t>
+          <t>Head hunter/HR Recruiter Senior - Fiumicino</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>EASYDIGITALGROUP</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -648,71 +648,67 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>Fiumicino, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=1204422a7ce9ec82</t>
+          <t>https://it.indeed.com/viewjob?jk=538bde2bee4e09c8</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Montatore/trice di arredi</t>
+          <t>Addetti alla selezione del personale</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>NETtoWORK</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Rome, Latium, Italy</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=3f6f3f6eef6c9b98</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2026-03-19</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4387906535</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Assuntore/trice rischi assicurativi junior</t>
+          <t>Contract Quality Intern</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>DocPlanner</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -722,32 +718,36 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Latina, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=713464501983a29f</t>
+          <t>https://it.indeed.com/viewjob?jk=b31c6859d3baff88</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Addetto/a Controllo Qualità</t>
+          <t>Project Analyst - Ecosistema Futuro</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>RONZONI GROUP STP STL SB</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Pomezia, LAZ, IT</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -765,7 +765,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=c5431c936083bcdb</t>
+          <t>https://it.indeed.com/viewjob?jk=9794cfdbbd68de5e</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -777,22 +777,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tecnico Collaudatore</t>
+          <t>Addetto/a Risorse Umane – Selezione e Formazione</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>EmmeBi Group</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Rome, Latium, Italy</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -800,34 +800,30 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=ee62bd4bd8d1da01</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>2026-03-19</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4387394112</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Expert business associate fluent in English and Italian</t>
+          <t>Addetto/a Risorse Umane - HR</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>To Be Service srl</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Rome, Latium, Italy</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -835,34 +831,34 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=cc8eb6e75904de4e</t>
+          <t>https://www.linkedin.com/jobs/view/4387120451</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Addetto/a alle Risorse Umane - UOS Gestione Rapporto di Lavoro</t>
+          <t>Operatore Elettrotermico</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Fondazione Policlinico Universitario Agostino Gemelli IRCCS</t>
+          <t>NTWK</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Rome, Latium, Italy</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -870,30 +866,34 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4387832543</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=c55d6bbd098a4b74</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HR Specialist – Selezione e Gestione Risorse Umane</t>
+          <t>Commerciali</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EmmeBi Group</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Rome, Latium, Italy</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -901,20 +901,24 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4387375901</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=1204422a7ce9ec82</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>HR Business Partner, EU One PXT</t>
+          <t>Montatore/trice di arredi</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -936,24 +940,24 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=ba09c547f83c23ae</t>
+          <t>https://it.indeed.com/viewjob?jk=3f6f3f6eef6c9b98</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Human Resources Director</t>
+          <t>Assuntore/trice rischi assicurativi junior</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Medici Senza Frontiere Onlus</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -963,19 +967,15 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Latina, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=f380e23a001e2d81</t>
+          <t>https://it.indeed.com/viewjob?jk=713464501983a29f</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -987,12 +987,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Executive Assistant Italy W/M</t>
+          <t>Addetto/a Controllo Qualità</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Fonroche Lighting</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Pomezia, LAZ, IT</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -1010,7 +1010,7 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=db5dbc790893673d</t>
+          <t>https://it.indeed.com/viewjob?jk=c5431c936083bcdb</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1022,12 +1022,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Intern</t>
+          <t>Tecnico Collaudatore</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Enza Zaden</t>
+          <t>NTWK</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1037,46 +1037,42 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Tarquinia, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>fulltime, internship</t>
-        </is>
-      </c>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=6d8507c16adc68ab</t>
+          <t>https://it.indeed.com/viewjob?jk=ee62bd4bd8d1da01</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Stagista risorse umane</t>
+          <t>Expert business associate fluent in English and Italian</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>REITHERA</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Rome, Latium, Italy</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -1084,34 +1080,34 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4386929399</t>
+          <t>https://it.indeed.com/viewjob?jk=cc8eb6e75904de4e</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>System Administration specialist full remote</t>
+          <t>Addetto/a alle Risorse Umane - UOS Gestione Rapporto di Lavoro</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>Fondazione Policlinico Universitario Agostino Gemelli IRCCS</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Rome, Latium, Italy</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -1119,34 +1115,30 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=481e24adc6ac754e</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4387832543</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Progettista Elettronico RF junior</t>
+          <t>HR Specialist – Selezione e Gestione Risorse Umane</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>EmmeBi Group</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Rome, Latium, Italy</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -1154,24 +1146,20 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=026e2987c6570a80</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4387375901</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Addetto/a Vendite profilo ESPERTO</t>
+          <t>HR Business Partner, EU One PXT</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1193,65 +1181,73 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=d57cf391056b87b2</t>
+          <t>https://it.indeed.com/viewjob?jk=ba09c547f83c23ae</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Impiegato/a Risorse Umane - Azienda settore moda</t>
+          <t>Human Resources Director</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>key-absolute</t>
+          <t>Medici Senza Frontiere Onlus</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Rieti, Latium, Italy</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4386862950</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=f380e23a001e2d81</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>HR Recruiter Assistant L.68/99 - Categoria Protetta Part Time</t>
+          <t>Executive Assistant Italy W/M</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BIP</t>
+          <t>Fonroche Lighting</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Rome, Latium, Italy</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -1259,90 +1255,98 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4387420383</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=db5dbc790893673d</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HR RECRUITER SPECIALIST</t>
+          <t>Intern</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>WJOB</t>
+          <t>Enza Zaden</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Rome, Latium, Italy</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
+          <t>Tarquinia, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>fulltime, internship</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4387283505</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=6d8507c16adc68ab</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>HR Business Partner, EU One PXT</t>
+          <t>Stagista risorse umane</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>REITHERA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Rome, Latium, Italy</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=4473aef4f50e8a6a</t>
+          <t>https://www.linkedin.com/jobs/view/4386929399</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>HR Compensation and Benefits</t>
+          <t>System Administration specialist full remote</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Fendi</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1360,24 +1364,24 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=c943fb245ebfa10e</t>
+          <t>https://it.indeed.com/viewjob?jk=481e24adc6ac754e</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Addetto/a Risorse Umane - HR</t>
+          <t>Progettista Elettronico RF junior</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Twins</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1390,16 +1394,12 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=f09d5e2b86de0ac3</t>
+          <t>https://it.indeed.com/viewjob?jk=026e2987c6570a80</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1411,43 +1411,51 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Junior Talent Acquisition Intern</t>
+          <t>Addetto/a Vendite profilo ESPERTO</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PQE Group</t>
+          <t>NTWK</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Rome, Latium, Italy</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4385019467</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=d57cf391056b87b2</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Talent Acquisition Specialist</t>
+          <t>Impiegato/a Risorse Umane - Azienda settore moda</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Openjobmetis SpA</t>
+          <t>key-absolute</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1457,7 +1465,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Aprilia, Latium, Italy</t>
+          <t>Rieti, Latium, Italy</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -1465,7 +1473,7 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4387117006</t>
+          <t>https://www.linkedin.com/jobs/view/4386862950</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -1473,12 +1481,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sales IT– Soluzioni AI &amp; Recruiting IT</t>
+          <t>HR Recruiter Assistant L.68/99 - Categoria Protetta Part Time</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Tron Group Holding</t>
+          <t>BIP</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1496,63 +1504,51 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4385385114</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4387420383</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cashier, Castel Romano, PT 18hr</t>
+          <t>HR RECRUITER SPECIALIST</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Michael Kors</t>
+          <t>WJOB</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>parttime</t>
-        </is>
-      </c>
+          <t>Rome, Latium, Italy</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=33a8dcee048685c5</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>2026-03-18</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4387283505</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Senior Human Resources Officer (Talent Acquisition)</t>
+          <t>HR Business Partner, EU One PXT</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Food and Agriculture Organization of the United Nations</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1565,29 +1561,33 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=900dbc9dfbe0fc1d</t>
+          <t>https://it.indeed.com/viewjob?jk=4473aef4f50e8a6a</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Senior Product Designer - Finance &amp; Reporting - 100% Remote - EMEA</t>
+          <t>HR Compensation and Benefits</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Hostaway</t>
+          <t>Fendi</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1600,113 +1600,109 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=32570765eeb92ac4</t>
+          <t>https://it.indeed.com/viewjob?jk=c943fb245ebfa10e</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Hr generalist appartenente alle categorie protette (art. 1 l. 68/99)</t>
+          <t>Addetto/a Risorse Umane - HR</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Ferrovie dello Stato Italiane S.p.A.</t>
+          <t>Twins</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Rome, Latium, Italy</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr"/>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4383335202</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=f09d5e2b86de0ac3</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Addetto/a Vendite profilo NEOFITA</t>
+          <t>Junior Talent Acquisition Intern</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>PQE Group</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>internship</t>
-        </is>
-      </c>
+          <t>Rome, Latium, Italy</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=3d77e742c3a1b0cf</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4385019467</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Operatore d’ufficio con competenze informatiche e CAD</t>
+          <t>Talent Acquisition Specialist</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>Openjobmetis SpA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Aprilia, Latium, Italy</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -1714,46 +1710,38 @@
       <c r="G36" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=07b89bd05a293ceb</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4387117006</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Addetto/a Vendite Pacchetti Turistici</t>
+          <t>Sales IT– Soluzioni AI &amp; Recruiting IT</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>Tron Group Holding</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Rome, Latium, Italy</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=d38789c4583fde1f</t>
+          <t>https://www.linkedin.com/jobs/view/4385385114</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -1765,12 +1753,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Responsabile Ufficio Calibrazione</t>
+          <t>Cashier, Castel Romano, PT 18hr</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>Michael Kors</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1783,29 +1771,33 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>parttime</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=cbbbd9ee3a0bf5fb</t>
+          <t>https://it.indeed.com/viewjob?jk=33a8dcee048685c5</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Tecnico specializzato (CND)</t>
+          <t>Senior Human Resources Officer (Talent Acquisition)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>Food and Agriculture Organization of the United Nations</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1815,7 +1807,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Rocca Priora, LAZ, IT</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -1823,24 +1815,24 @@
       <c r="G39" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=f0058b00836b6aab</t>
+          <t>https://it.indeed.com/viewjob?jk=900dbc9dfbe0fc1d</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Payroll Specialist</t>
+          <t>Senior Product Designer - Finance &amp; Reporting - 100% Remote - EMEA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Gruppo Paoletti</t>
+          <t>Hostaway</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1850,7 +1842,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Fiumicino, LAZ, IT</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1862,34 +1854,34 @@
       <c r="G40" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=a20837d2f68ef361</t>
+          <t>https://it.indeed.com/viewjob?jk=32570765eeb92ac4</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Export Specialist (Air Freight)</t>
+          <t>Hr generalist appartenente alle categorie protette (art. 1 l. 68/99)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Crane Worldwide Logistics</t>
+          <t>Ferrovie dello Stato Italiane S.p.A.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Fiumicino, LAZ, IT</t>
+          <t>Rome, Latium, Italy</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -1897,19 +1889,15 @@
       <c r="G41" t="inlineStr"/>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=3f8cbae858d8f03c</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4383335202</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Addetto/a Front Office</t>
+          <t>Addetto/a Vendite profilo NEOFITA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1924,19 +1912,19 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Frosinone, LAZ, IT</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>fulltime</t>
+          <t>internship</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=43d7d4d0625f532a</t>
+          <t>https://it.indeed.com/viewjob?jk=3d77e742c3a1b0cf</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -1948,7 +1936,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ASPP</t>
+          <t>Operatore d’ufficio con competenze informatiche e CAD</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1971,7 +1959,7 @@
       <c r="G43" t="inlineStr"/>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=ca6a36c647f60db8</t>
+          <t>https://it.indeed.com/viewjob?jk=07b89bd05a293ceb</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -1983,7 +1971,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Assistente Commerciale</t>
+          <t>Addetto/a Vendite Pacchetti Turistici</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1998,19 +1986,19 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Frosinone, LAZ, IT</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>parttime, fulltime</t>
+          <t>fulltime</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=bc72aa3f759a220e</t>
+          <t>https://it.indeed.com/viewjob?jk=d38789c4583fde1f</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2022,12 +2010,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Specialista HSE</t>
+          <t>Responsabile Ufficio Calibrazione</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2045,7 +2033,7 @@
       <c r="G45" t="inlineStr"/>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=96fec7b622be5064</t>
+          <t>https://it.indeed.com/viewjob?jk=cbbbd9ee3a0bf5fb</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2057,22 +2045,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Stagista risorse umane</t>
+          <t>Tecnico specializzato (CND)</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Sibylla S.r.l.</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Rome, Latium, Italy</t>
+          <t>Rocca Priora, LAZ, IT</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -2080,61 +2068,73 @@
       <c r="G46" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4386917955</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=f0058b00836b6aab</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Responsabile Risorse Umane</t>
+          <t>Payroll Specialist</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>EmmeBi Group</t>
+          <t>Gruppo Paoletti</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Ferentino, Latium, Italy</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr"/>
+          <t>Fiumicino, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4385907928</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=a20837d2f68ef361</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Impiegato/a Risorse Umane - Grande Distribuzione Organizzata</t>
+          <t>Export Specialist (Air Freight)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>tecno-system</t>
+          <t>Crane Worldwide Logistics</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Anagni, Latium, Italy</t>
+          <t>Fiumicino, LAZ, IT</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -2142,57 +2142,73 @@
       <c r="G48" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4385912724</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=3f8cbae858d8f03c</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Recruiter Trainee</t>
+          <t>Addetto/a Front Office</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Chaberton Professionals</t>
+          <t>NTWK</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Frosinone, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4384496823</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=43d7d4d0625f532a</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>HR Recruiter</t>
+          <t>ASPP</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Openjobmetis SpA</t>
+          <t>NTWK</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Ariccia, Latium, Italy</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -2200,20 +2216,24 @@
       <c r="G50" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4385953009</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=ca6a36c647f60db8</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>HR Business Partner, EU One PXT</t>
+          <t>Assistente Commerciale</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>NTWK</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2223,36 +2243,36 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Frosinone, LAZ, IT</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>fulltime</t>
+          <t>parttime, fulltime</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=710888b0f40062e5</t>
+          <t>https://it.indeed.com/viewjob?jk=bc72aa3f759a220e</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>IMPIEGATO AMMINISTRATIVO RISORSE UMANE – AREA OPERATIVA</t>
+          <t>Specialista HSE</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CRI Roma</t>
+          <t>NTWK</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2265,16 +2285,12 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=9e7cce514343f0dd</t>
+          <t>https://it.indeed.com/viewjob?jk=96fec7b622be5064</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2286,51 +2302,43 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>P&amp;C Intern - Personal Administration</t>
+          <t>Stagista risorse umane</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Philip Morris International</t>
+          <t>Sibylla S.r.l.</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Rome, Latium, Italy</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=776e59d8a9befd96</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4386917955</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>HR / Talent Acquisition Specialist – Tutor per lezioni private</t>
+          <t>Responsabile Risorse Umane</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Letuelezioni</t>
+          <t>EmmeBi Group</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2338,13 +2346,17 @@
           <t>linkedin</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Ferentino, Latium, Italy</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4385972264</t>
+          <t>https://www.linkedin.com/jobs/view/4385907928</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -2352,12 +2364,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>HR Administration (Risorse umane)</t>
+          <t>Impiegato/a Risorse Umane - Grande Distribuzione Organizzata</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Joinrs</t>
+          <t>tecno-system</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2367,7 +2379,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Rome, Latium, Italy</t>
+          <t>Anagni, Latium, Italy</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -2375,7 +2387,7 @@
       <c r="G55" t="inlineStr"/>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4386305987</t>
+          <t>https://www.linkedin.com/jobs/view/4385912724</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -2383,61 +2395,49 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Fitness Partners Executive</t>
+          <t>Recruiter Trainee</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Wellhub</t>
+          <t>Chaberton Professionals</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>indeed</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>parttime, internship</t>
-        </is>
-      </c>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=e872b6a8d69aca4b</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>2026-03-16</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4384496823</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Senior Audit Public - Roma</t>
+          <t>HR Recruiter</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>BDO</t>
+          <t>Openjobmetis SpA</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Ariccia, Latium, Italy</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -2445,24 +2445,20 @@
       <c r="G57" t="inlineStr"/>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=39acb4f121d0779d</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>2026-03-16</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4385953009</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>IT Jira Specialist</t>
+          <t>HR Business Partner, EU One PXT</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2475,29 +2471,33 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=29a20dacb25e8c67</t>
+          <t>https://it.indeed.com/viewjob?jk=710888b0f40062e5</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Ingegnere Gestionale / Ingegnere Civile – Gestione Commesse &amp; Sistemi ERP</t>
+          <t>IMPIEGATO AMMINISTRATIVO RISORSE UMANE – AREA OPERATIVA</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>CRI Roma</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2510,29 +2510,33 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=f771facb3974b4fd</t>
+          <t>https://it.indeed.com/viewjob?jk=9e7cce514343f0dd</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Addetto/a servizi mensa</t>
+          <t>P&amp;C Intern - Personal Administration</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>NHRG SRL – Agenzia per il Lavoro</t>
+          <t>Philip Morris International</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2542,81 +2546,73 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Rieti, LAZ, IT</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>parttime</t>
+          <t>fulltime</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=c00a2ade3b4e5aa8</t>
+          <t>https://it.indeed.com/viewjob?jk=776e59d8a9befd96</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Addetto/a Ufficio Ordini</t>
+          <t>HR / Talent Acquisition Specialist – Tutor per lezioni private</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>Letuelezioni</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>indeed</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=42e6ac7f25423163</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>2026-03-16</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4385972264</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>DISPONENTE / IMPIEGATO OPERATIVO TRASPORTI</t>
+          <t>HR Administration (Risorse umane)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>Joinrs</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Rome, Latium, Italy</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -2624,24 +2620,20 @@
       <c r="G62" t="inlineStr"/>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=e474b628bc63e59b</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>2026-03-16</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4386305987</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Progettista unità di potenza</t>
+          <t>Fitness Partners Executive</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>Wellhub</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2654,12 +2646,16 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>parttime, internship</t>
+        </is>
+      </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=9a902068a34038ea</t>
+          <t>https://it.indeed.com/viewjob?jk=e872b6a8d69aca4b</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -2671,12 +2667,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Security analyst</t>
+          <t>Senior Audit Public - Roma</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>BDO</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2694,7 +2690,7 @@
       <c r="G64" t="inlineStr"/>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=1c091c6b7a66e8d4</t>
+          <t>https://it.indeed.com/viewjob?jk=39acb4f121d0779d</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -2706,12 +2702,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>HR Business Partner, EU One PXT</t>
+          <t>IT Jira Specialist</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2724,33 +2720,29 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=a129e177a751dd36</t>
+          <t>https://it.indeed.com/viewjob?jk=29a20dacb25e8c67</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>HR Generalist</t>
+          <t>Ingegnere Gestionale / Ingegnere Civile – Gestione Commesse &amp; Sistemi ERP</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2768,7 +2760,7 @@
       <c r="G66" t="inlineStr"/>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=3aa7e72976109c1d</t>
+          <t>https://it.indeed.com/viewjob?jk=f771facb3974b4fd</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -2780,12 +2772,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>People Business Partner and Administration Specialist - Fixed term (1 year contract)</t>
+          <t>Addetto/a servizi mensa</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>NHRG SRL – Agenzia per il Lavoro</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2795,15 +2787,19 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Caprarola, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr"/>
+          <t>Rieti, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>parttime</t>
+        </is>
+      </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=f2d21dab4e62346a</t>
+          <t>https://it.indeed.com/viewjob?jk=c00a2ade3b4e5aa8</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -2815,12 +2811,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Addetto/a Area Risorse Umane - Gestione del Personale</t>
+          <t>Addetto/a Ufficio Ordini</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Cosma solution</t>
+          <t>NTWK</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2830,19 +2826,15 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Frosinone, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=84348e9491ac125d</t>
+          <t>https://it.indeed.com/viewjob?jk=42e6ac7f25423163</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -2854,22 +2846,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Ayvens Recruiting Day – Marzo 2026 Roma</t>
+          <t>DISPONENTE / IMPIEGATO OPERATIVO TRASPORTI</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Ayvens</t>
+          <t>NTWK</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Rome, Latium, Italy</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -2877,20 +2869,24 @@
       <c r="G69" t="inlineStr"/>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4384440393</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=e474b628bc63e59b</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Senior Sales Consultant (formazione e consulenza HR)</t>
+          <t>Progettista unità di potenza</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Randstad</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2900,19 +2896,15 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=b921857b4f137665</t>
+          <t>https://it.indeed.com/viewjob?jk=9a902068a34038ea</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -2924,12 +2916,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>HR Business Partner, EU One PXT</t>
+          <t>Security analyst</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2942,33 +2934,29 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=77501ea08c1b0f0b</t>
+          <t>https://it.indeed.com/viewjob?jk=1c091c6b7a66e8d4</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Ingegnere/Architetto Tender Specialist</t>
+          <t>HR Business Partner, EU One PXT</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Saturno Consulting HR</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2990,24 +2978,24 @@
       <c r="G72" t="inlineStr"/>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=057f40c23a96b33b</t>
+          <t>https://it.indeed.com/viewjob?jk=a129e177a751dd36</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Optical Technical Project Manager</t>
+          <t>HR Generalist</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Terna</t>
+          <t>NTWK</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3025,24 +3013,24 @@
       <c r="G73" t="inlineStr"/>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=41451cf3b33375bb</t>
+          <t>https://it.indeed.com/viewjob?jk=3aa7e72976109c1d</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Ingegnere Meccanico DL e Progettazione</t>
+          <t>People Business Partner and Administration Specialist - Fixed term (1 year contract)</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Saturno Consulting HR</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3052,36 +3040,32 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Caprarola, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=e35f0347ad252e7e</t>
+          <t>https://it.indeed.com/viewjob?jk=f2d21dab4e62346a</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Project Planner e Controller</t>
+          <t>Addetto/a Area Risorse Umane - Gestione del Personale</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Terna</t>
+          <t>Cosma solution</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3091,71 +3075,67 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr"/>
+          <t>Frosinone, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=2a33a0c2a06a8a50</t>
+          <t>https://it.indeed.com/viewjob?jk=84348e9491ac125d</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Direttore Tecnico Cantieri Verde Pubblico</t>
+          <t>Ayvens Recruiting Day – Marzo 2026 Roma</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Saturno Consulting HR</t>
+          <t>Ayvens</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Rome, Latium, Italy</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=5a47745206230804</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>2026-03-15</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4384440393</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Area Manager, FC Operations</t>
+          <t>Senior Sales Consultant (formazione e consulenza HR)</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>Randstad</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3165,7 +3145,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Passo Corese, LAZ, IT</t>
+          <t>LAZ, IT</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3177,19 +3157,19 @@
       <c r="G77" t="inlineStr"/>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=86f0a0a875b60568</t>
+          <t>https://it.indeed.com/viewjob?jk=b921857b4f137665</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-03-16</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Military - Area Manager - Italy</t>
+          <t>HR Business Partner, EU One PXT</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3204,7 +3184,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Colleferro, LAZ, IT</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3216,24 +3196,24 @@
       <c r="G78" t="inlineStr"/>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=8e8a6819a3bfb95c</t>
+          <t>https://it.indeed.com/viewjob?jk=77501ea08c1b0f0b</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Senior SAP BTP &amp; AI Architect</t>
+          <t>Ingegnere/Architetto Tender Specialist</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Saturno Consulting HR</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3255,7 +3235,7 @@
       <c r="G79" t="inlineStr"/>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=ee4ec82da870e1de</t>
+          <t>https://it.indeed.com/viewjob?jk=057f40c23a96b33b</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -3267,12 +3247,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>HR Business Partner, EU One PXT</t>
+          <t>Optical Technical Project Manager</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>Terna</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3285,33 +3265,29 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=056e07e3d7c45fe7</t>
+          <t>https://it.indeed.com/viewjob?jk=41451cf3b33375bb</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-09</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Animatore turistico/animatrice turistica</t>
+          <t>Ingegnere Meccanico DL e Progettazione</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Entertainment Dance</t>
+          <t>Saturno Consulting HR</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3321,36 +3297,36 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Viterbo, LAZ, IT</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>parttime, fulltime</t>
+          <t>fulltime</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=9e882f75a5617d9a</t>
+          <t>https://it.indeed.com/viewjob?jk=e35f0347ad252e7e</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-15</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Event Manager</t>
+          <t>Project Planner e Controller</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Cento per Centro S.r.l.</t>
+          <t>Terna</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3360,19 +3336,15 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Rieti, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>parttime</t>
-        </is>
-      </c>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=fb648027dd3021c7</t>
+          <t>https://it.indeed.com/viewjob?jk=2a33a0c2a06a8a50</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -3384,12 +3356,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Area Manager, FC Operations</t>
+          <t>Direttore Tecnico Cantieri Verde Pubblico</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>Saturno Consulting HR</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3399,7 +3371,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Passo Corese, LAZ, IT</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3411,19 +3383,19 @@
       <c r="G83" t="inlineStr"/>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=49235986d2cf6301</t>
+          <t>https://it.indeed.com/viewjob?jk=5a47745206230804</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-03-15</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Military - Area Manager - Italy</t>
+          <t>Area Manager, FC Operations</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3438,7 +3410,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Colleferro, LAZ, IT</t>
+          <t>Passo Corese, LAZ, IT</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3450,19 +3422,19 @@
       <c r="G84" t="inlineStr"/>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=bd1b3e59c44ec5bb</t>
+          <t>https://it.indeed.com/viewjob?jk=86f0a0a875b60568</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-01-28</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>HR Business Partner, EU One PXT</t>
+          <t>Military - Area Manager - Italy</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3477,7 +3449,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Colleferro, LAZ, IT</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3489,50 +3461,58 @@
       <c r="G85" t="inlineStr"/>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=451c1165395cdd9c</t>
+          <t>https://it.indeed.com/viewjob?jk=8e8a6819a3bfb95c</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-02-20</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>LUISS meets Generali - Recruiting Day</t>
+          <t>Senior SAP BTP &amp; AI Architect</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Agenzia Generali Roma Corso Trieste</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Rome, Latium, Italy</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr"/>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4383639535</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=ee4ec82da870e1de</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Area Manager, FC Operations</t>
+          <t>HR Business Partner, EU One PXT</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3547,7 +3527,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Passo Corese, LAZ, IT</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -3559,24 +3539,24 @@
       <c r="G87" t="inlineStr"/>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=22a1ddf420e0d824</t>
+          <t>https://it.indeed.com/viewjob?jk=056e07e3d7c45fe7</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Military - Area Manager - Italy</t>
+          <t>Animatore turistico/animatrice turistica</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>Entertainment Dance</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3586,36 +3566,36 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Colleferro, LAZ, IT</t>
+          <t>Viterbo, LAZ, IT</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>fulltime</t>
+          <t>parttime, fulltime</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=e6cf390409a2cf78</t>
+          <t>https://it.indeed.com/viewjob?jk=9e882f75a5617d9a</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-03-14</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HR Business Partner, EU One PXT</t>
+          <t>Event Manager</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>Cento per Centro S.r.l.</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3625,36 +3605,36 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Rieti, LAZ, IT</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>fulltime</t>
+          <t>parttime</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=727f9bebb7430afb</t>
+          <t>https://it.indeed.com/viewjob?jk=fb648027dd3021c7</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-10</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Addetto/a vendite Part time - Outlet Castel Romano</t>
+          <t>Area Manager, FC Operations</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Skechers</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3664,36 +3644,36 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Passo Corese, LAZ, IT</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>parttime</t>
+          <t>fulltime</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=f96e50d1e6879e04</t>
+          <t>https://it.indeed.com/viewjob?jk=49235986d2cf6301</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-01-28</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Addetto/a all’ufficio avanzamento del Centro di Eccellenza Meccanico</t>
+          <t>Military - Area Manager - Italy</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Leonardo</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3703,32 +3683,36 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Cisterna di Latina, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr"/>
+          <t>Colleferro, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=66b8c7691cd359f2</t>
+          <t>https://it.indeed.com/viewjob?jk=bd1b3e59c44ec5bb</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-02-20</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Responsabile Technical Procurement</t>
+          <t>HR Business Partner, EU One PXT</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ITA airways</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3738,42 +3722,46 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Fiumicino, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr"/>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=99039b787e45436a</t>
+          <t>https://it.indeed.com/viewjob?jk=451c1165395cdd9c</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>MEDICO DI REPARTO - M/F</t>
+          <t>LUISS meets Generali - Recruiting Day</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>KORIAN</t>
+          <t>Agenzia Generali Roma Corso Trieste</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Campagnano di Roma, LAZ, IT</t>
+          <t>Rome, Latium, Italy</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -3781,24 +3769,20 @@
       <c r="G93" t="inlineStr"/>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=72afea7f6212e0e6</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4383639535</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Progettista meccanico</t>
+          <t>Area Manager, FC Operations</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>PROGER</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -3808,7 +3792,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Passo Corese, LAZ, IT</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -3820,24 +3804,24 @@
       <c r="G94" t="inlineStr"/>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=155bafc2ad9a4f55</t>
+          <t>https://it.indeed.com/viewjob?jk=22a1ddf420e0d824</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-01-28</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Assistente al Coordinatore Clinico</t>
+          <t>Military - Area Manager - Italy</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Tutti giù per terra Onlus</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -3847,32 +3831,36 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr"/>
+          <t>Colleferro, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=353770ee335e013b</t>
+          <t>https://it.indeed.com/viewjob?jk=e6cf390409a2cf78</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-02-20</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Stagista Help Desk - Roma</t>
+          <t>HR Business Partner, EU One PXT</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>BONELLI EREDE PAPPALARDO</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3887,31 +3875,31 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>internship</t>
+          <t>fulltime</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=27b3108f7567db7a</t>
+          <t>https://it.indeed.com/viewjob?jk=727f9bebb7430afb</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-05</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Addetti alle vendite</t>
+          <t>Addetto/a vendite Part time - Outlet Castel Romano</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Pilato Store</t>
+          <t>Skechers</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3926,14 +3914,14 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>parttime, fulltime</t>
+          <t>parttime</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr"/>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=4f9917c9f4eff5f9</t>
+          <t>https://it.indeed.com/viewjob?jk=f96e50d1e6879e04</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -3945,10 +3933,14 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Responsabile Di Negozio</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr"/>
+          <t>Addetto/a all’ufficio avanzamento del Centro di Eccellenza Meccanico</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Leonardo</t>
+        </is>
+      </c>
       <c r="C98" t="inlineStr">
         <is>
           <t>indeed</t>
@@ -3956,7 +3948,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Cisterna di Latina, LAZ, IT</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -3964,7 +3956,7 @@
       <c r="G98" t="inlineStr"/>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=ff5fafbeb3752b08</t>
+          <t>https://it.indeed.com/viewjob?jk=66b8c7691cd359f2</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -3976,12 +3968,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Architetto Infrastrutturale</t>
+          <t>Responsabile Technical Procurement</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>NETwk</t>
+          <t>ITA airways</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3991,7 +3983,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Fiumicino, LAZ, IT</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -3999,7 +3991,7 @@
       <c r="G99" t="inlineStr"/>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=215e2625f80dfca1</t>
+          <t>https://it.indeed.com/viewjob?jk=99039b787e45436a</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -4011,12 +4003,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Addetto/a servizi mensa</t>
+          <t>MEDICO DI REPARTO - M/F</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>NHRG SRL – Agenzia per il Lavoro</t>
+          <t>KORIAN</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4026,19 +4018,15 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Rieti, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>parttime</t>
-        </is>
-      </c>
+          <t>Campagnano di Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr"/>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=2f63182ded1e797e</t>
+          <t>https://it.indeed.com/viewjob?jk=72afea7f6212e0e6</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -4050,12 +4038,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Junior PMO Pubblica Amministrazione</t>
+          <t>Progettista meccanico</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>BDO</t>
+          <t>PROGER</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4068,12 +4056,16 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=56f8f83b3dbc221e</t>
+          <t>https://it.indeed.com/viewjob?jk=155bafc2ad9a4f55</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -4085,12 +4077,12 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Animatori per bambini e ragazzi in soggiorni residenziali</t>
+          <t>Assistente al Coordinatore Clinico</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>DOC s.c.s.</t>
+          <t>Tutti giù per terra Onlus</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4103,33 +4095,29 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=2379cce56a434871</t>
+          <t>https://it.indeed.com/viewjob?jk=353770ee335e013b</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Lavoro a ROMA - COLLOQUIO IN sede BARBERINI</t>
+          <t>Stagista Help Desk - Roma</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Globe MKD</t>
+          <t>BONELLI EREDE PAPPALARDO</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4142,29 +4130,33 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>internship</t>
+        </is>
+      </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr"/>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=5ca7c4c08a45923f</t>
+          <t>https://it.indeed.com/viewjob?jk=27b3108f7567db7a</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-12</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Addetti alle vendite</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Terna</t>
+          <t>Pilato Store</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4177,12 +4169,16 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>parttime, fulltime</t>
+        </is>
+      </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=b05d2a6aa42288f0</t>
+          <t>https://it.indeed.com/viewjob?jk=4f9917c9f4eff5f9</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -4194,22 +4190,18 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Impiegato/a Risorse Umane | Consulenze</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>key-absolute</t>
-        </is>
-      </c>
+          <t>Responsabile Di Negozio</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Rome, Latium, Italy</t>
+          <t>Roma, LAZ, IT</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -4217,20 +4209,24 @@
       <c r="G105" t="inlineStr"/>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4384261319</t>
-        </is>
-      </c>
-      <c r="I105" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=ff5fafbeb3752b08</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Area Manager, FC Operations</t>
+          <t>Architetto Infrastrutturale</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>NETwk</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -4240,36 +4236,32 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Passo Corese, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=9458a38ff98817fa</t>
+          <t>https://it.indeed.com/viewjob?jk=215e2625f80dfca1</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-03-13</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Military - Area Manager - Italy</t>
+          <t>Addetto/a servizi mensa</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>NHRG SRL – Agenzia per il Lavoro</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -4279,36 +4271,36 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Colleferro, LAZ, IT</t>
+          <t>Rieti, LAZ, IT</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>fulltime</t>
+          <t>parttime</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr"/>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=a51f253cfb43e8ad</t>
+          <t>https://it.indeed.com/viewjob?jk=2f63182ded1e797e</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-03-13</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Programme Officer – Global Rapid Response Team (Access &amp; HMI Specialist)</t>
+          <t>Junior PMO Pubblica Amministrazione</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>World Food Programme</t>
+          <t>BDO</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -4321,16 +4313,12 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr"/>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=2b0c5fc77486f46c</t>
+          <t>https://it.indeed.com/viewjob?jk=56f8f83b3dbc221e</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -4342,12 +4330,12 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Junior School Class Teacher</t>
+          <t>Animatori per bambini e ragazzi in soggiorni residenziali</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>St George's British International School</t>
+          <t>DOC s.c.s.</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -4369,7 +4357,7 @@
       <c r="G109" t="inlineStr"/>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=2e3868f91731b8bc</t>
+          <t>https://it.indeed.com/viewjob?jk=2379cce56a434871</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -4381,12 +4369,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>HR Business Partner, EU One PXT</t>
+          <t>Lavoro a ROMA - COLLOQUIO IN sede BARBERINI</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Amazon.com</t>
+          <t>Globe MKD</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -4399,33 +4387,29 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=64a42c84f116d4d6</t>
+          <t>https://it.indeed.com/viewjob?jk=5ca7c4c08a45923f</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-13</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>HR Generalist (Categorie Protette L.68/99)</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>FILMMASTER</t>
+          <t>Terna</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4438,16 +4422,12 @@
           <t>Roma, LAZ, IT</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+      <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr"/>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=9bb6d72ced10d28a</t>
+          <t>https://it.indeed.com/viewjob?jk=b05d2a6aa42288f0</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -4459,82 +4439,82 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>HR Clerk - maternity cover</t>
+          <t>Impiegato/a Risorse Umane | Consulenze</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Abbott</t>
+          <t>key-absolute</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Rome, Latium, Italy</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr"/>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>https://it.indeed.com/viewjob?jk=cf06994c867d9dde</t>
-        </is>
-      </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4384261319</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>CLIENT RECRUITMENT SPECIALIST ON SITE</t>
+          <t>Area Manager, FC Operations</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Gi Group</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Rome, Latium, Italy</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr"/>
+          <t>Passo Corese, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr"/>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4383146711</t>
-        </is>
-      </c>
-      <c r="I113" t="inlineStr"/>
+          <t>https://it.indeed.com/viewjob?jk=9458a38ff98817fa</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>HR Talent Support Intern</t>
+          <t>Military - Area Manager - Italy</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Ayvens</t>
+          <t>Amazon.com</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -4544,7 +4524,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Roma, LAZ, IT</t>
+          <t>Colleferro, LAZ, IT</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -4556,17 +4536,282 @@
       <c r="G114" t="inlineStr"/>
       <c r="H114" s="2" t="inlineStr">
         <is>
+          <t>https://it.indeed.com/viewjob?jk=a51f253cfb43e8ad</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Programme Officer – Global Rapid Response Team (Access &amp; HMI Specialist)</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>World Food Programme</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>https://it.indeed.com/viewjob?jk=2b0c5fc77486f46c</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Junior School Class Teacher</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>St George's British International School</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>https://it.indeed.com/viewjob?jk=2e3868f91731b8bc</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>HR Business Partner, EU One PXT</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Amazon.com</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>https://it.indeed.com/viewjob?jk=64a42c84f116d4d6</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>HR Generalist (Categorie Protette L.68/99)</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>FILMMASTER</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>https://it.indeed.com/viewjob?jk=9bb6d72ced10d28a</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>HR Clerk - maternity cover</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Abbott</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>https://it.indeed.com/viewjob?jk=cf06994c867d9dde</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>CLIENT RECRUITMENT SPECIALIST ON SITE</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Gi Group</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Rome, Latium, Italy</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4383146711</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>HR Talent Support Intern</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Ayvens</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Roma, LAZ, IT</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
           <t>https://it.indeed.com/viewjob?jk=1893b6c166669e55</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr">
+      <c r="I121" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I114"/>
+  <autoFilter ref="A1:I121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>